<commit_message>
Added feature to validate DB vs Excel/CSV
</commit_message>
<xml_diff>
--- a/output/comparison-report.xlsx
+++ b/output/comparison-report.xlsx
@@ -81,7 +81,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Expected File</t>
+          <t>Expected Source</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -117,7 +117,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="9">
@@ -157,7 +157,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="13">
@@ -190,7 +190,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -201,7 +201,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -236,6 +236,102 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>HEADER_MISMATCH</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>sfasdfds</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>EXTRA</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Extra header in actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>HEADER_MISMATCH</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>sadfwe3</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>EXTRA</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Extra header in actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>VALUE_MISMATCH</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TEST-REFUND-OVER</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Transaction Type</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>purddchase</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>purchase</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Text values differ after configured normalization</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>